<commit_message>
Stage 2 v3: clarify target-achieved figures and record known defect
Replace the headline 'utilization target achieved 40 / 40' in the v3 README,
VERSIONS.md and sheet 1 of the v1/v2/v3 workbook with two figures: target
achieved where the baseline was overloaded (>0.85): 25 of 25; all 40
utilization runs: 40 of 40, of which 15 already below 0.85 at baseline.
Record the known defect: direction filter reads KPI name instead of category
(affects Procure2Pay_G3 only; baseline already below 0.85; no score change; to
be fixed in the next version).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evaluation/loanapp_p2p/results/GLASS_Stage2_results_v1_v2_v3.xlsx
+++ b/evaluation/loanapp_p2p/results/GLASS_Stage2_results_v1_v2_v3.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1434,12 +1434,12 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>target achieved where the baseline was overloaded (&gt;0.85): 25 of 25; all 40 utilization runs: 40 of 40, of which 15 already below 0.85 at baseline</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>target achieved where the baseline was overloaded (&gt;0.85): 25 of 25; all 40 utilization runs: 40 of 40, of which 15 already below 0.85 at baseline</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>target achieved where the baseline was overloaded (&gt;0.85): 25 of 25; all 40 utilization runs: 40 of 40, of which 15 already below 0.85 at baseline</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>target achieved where the baseline was overloaded (&gt;0.85): 25 of 25; all 40 utilization runs: 40 of 40, of which 15 already below 0.85 at baseline</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Direction filter (v3): it reads the metric from the KPI name, so for the three utilization KPIs without "utilization" in their name nothing was filtered; in Procure2Pay_G3 (12 feedback texts) strategies raising utilization were still shown. See VERSIONS.md and the v3 README.</t>
+          <t>Utilization target achieved (v3, after refinement): target achieved where the baseline was overloaded (&gt;0.85): 25 of 25; all 40 utilization runs: 40 of 40, of which 15 already below 0.85 at baseline. Both figures hold under GLASS's flag (at most 0.85) and under our rule (below 0.85).</t>
         </is>
       </c>
       <c r="B22" s="4" t="n"/>
@@ -1659,7 +1659,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Runs affected by the unit defect (v1 / v2): a proposed duration meant in hours was applied in seconds. Their scores are kept as recorded and are included in all counts (see VERSIONS.md). v3 rejects such modifications.</t>
+          <t>Known defect: direction filter reads KPI name instead of category (affects Procure2Pay_G3 only; baseline already below 0.85; no score change; to be fixed in the next version).</t>
         </is>
       </c>
       <c r="B23" s="4" t="n"/>
@@ -1677,7 +1677,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Source: stage2_v1_v2_v3.csv (from the verified per-configuration and summary CSVs of the three batches).</t>
+          <t>Runs affected by the unit defect (v1 / v2): a proposed duration meant in hours was applied in seconds. Their scores are kept as recorded and are included in all counts (see VERSIONS.md). v3 rejects such modifications.</t>
         </is>
       </c>
       <c r="B24" s="4" t="n"/>
@@ -1693,7 +1693,11 @@
       <c r="L24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Source: stage2_v1_v2_v3.csv (from the verified per-configuration and summary CSVs of the three batches).</t>
+        </is>
+      </c>
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
@@ -1707,11 +1711,7 @@
       <c r="L25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Change from v2 to v3 per group (v3 − v2)</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="n"/>
       <c r="B26" s="4" t="n"/>
       <c r="C26" s="4" t="n"/>
       <c r="D26" s="4" t="n"/>
@@ -1725,41 +1725,17 @@
       <c r="L26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Valid scenario (after refinement)</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>All target KPIs improved, our rule (after refinement)</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Valid and all KPIs improved, our rule (after refinement)</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Runs where the refinement made the result worse</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>Share of injected changes recovered (after refinement)</t>
-        </is>
-      </c>
-      <c r="G27" s="1" t="inlineStr">
-        <is>
-          <t>Closeness to the healthy model, median (after refinement)</t>
-        </is>
-      </c>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Change from v2 to v3 per group (v3 − v2)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
       <c r="J27" s="4" t="n"/>
@@ -1767,39 +1743,39 @@
       <c r="L27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>With a utilization KPI</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>+16</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>+16</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>+5</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>+0.028</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>+0.026</t>
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Valid scenario (after refinement)</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>All target KPIs improved, our rule (after refinement)</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>Valid and all KPIs improved, our rule (after refinement)</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Runs where the refinement made the result worse</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>Share of injected changes recovered (after refinement)</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>Closeness to the healthy model, median (after refinement)</t>
         </is>
       </c>
       <c r="H28" s="4" t="n"/>
@@ -1811,37 +1787,37 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Without a utilization KPI (control)</t>
+          <t>With a utilization KPI</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+16</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+16</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>-0.015</t>
+          <t>+0.028</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>-0.005</t>
+          <t>+0.026</t>
         </is>
       </c>
       <c r="H29" s="4" t="n"/>
@@ -1851,13 +1827,41 @@
       <c r="L29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Without a utilization KPI (control)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>-0.015</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>-0.005</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
@@ -1865,11 +1869,7 @@
       <c r="L30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Change from v1 to v3 per group (v3 − v1)</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="n"/>
       <c r="B31" s="4" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="4" t="n"/>
@@ -1883,41 +1883,17 @@
       <c r="L31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>Valid scenario (after refinement)</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>All target KPIs improved, our rule (after refinement)</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="inlineStr">
-        <is>
-          <t>Valid and all KPIs improved, our rule (after refinement)</t>
-        </is>
-      </c>
-      <c r="E32" s="1" t="inlineStr">
-        <is>
-          <t>Runs where the refinement made the result worse</t>
-        </is>
-      </c>
-      <c r="F32" s="1" t="inlineStr">
-        <is>
-          <t>Share of injected changes recovered (after refinement)</t>
-        </is>
-      </c>
-      <c r="G32" s="1" t="inlineStr">
-        <is>
-          <t>Closeness to the healthy model, median (after refinement)</t>
-        </is>
-      </c>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Change from v1 to v3 per group (v3 − v1)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
       <c r="J32" s="4" t="n"/>
@@ -1925,39 +1901,39 @@
       <c r="L32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>With a utilization KPI</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>+0</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>+17</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>+17</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>-8</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>+0.030</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>+0.480</t>
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>Valid scenario (after refinement)</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>All target KPIs improved, our rule (after refinement)</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>Valid and all KPIs improved, our rule (after refinement)</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Runs where the refinement made the result worse</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>Share of injected changes recovered (after refinement)</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>Closeness to the healthy model, median (after refinement)</t>
         </is>
       </c>
       <c r="H33" s="4" t="n"/>
@@ -1969,37 +1945,37 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Without a utilization KPI (control)</t>
+          <t>With a utilization KPI</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+0</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>+17</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>+17</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>-0.018</t>
+          <t>+0.030</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>-0.038</t>
+          <t>+0.480</t>
         </is>
       </c>
       <c r="H34" s="4" t="n"/>
@@ -2009,13 +1985,41 @@
       <c r="L34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Without a utilization KPI (control)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>-3</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>-6</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>-0.018</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>-0.038</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="n"/>
@@ -2023,11 +2027,7 @@
       <c r="L35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Control check v1 → v2</t>
-        </is>
-      </c>
+      <c r="A36" s="4" t="n"/>
       <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="n"/>
       <c r="D36" s="4" t="n"/>
@@ -2041,9 +2041,9 @@
       <c r="L36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Sign test over the 6 configurations: 4 differ, 1 of them higher in v2; two-sided p = 0.625.</t>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Control check v1 → v2</t>
         </is>
       </c>
       <c r="B37" s="4" t="n"/>
@@ -2061,7 +2061,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Pooled run-level Fisher exact test: 23/30 in v1 vs 20/30 in v2; p = 0.567.</t>
+          <t>Sign test over the 6 configurations: 4 differ, 1 of them higher in v2; two-sided p = 0.625.</t>
         </is>
       </c>
       <c r="B38" s="4" t="n"/>
@@ -2079,7 +2079,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Reading: the control configurations are statistically indistinguishable between v1 and v2 at the 5 % level. With 6 configurations, the sign test can detect only large systematic shifts. The LLM is not seeded, so run-to-run variation alone also differs between versions.</t>
+          <t>Pooled run-level Fisher exact test: 23/30 in v1 vs 20/30 in v2; p = 0.567.</t>
         </is>
       </c>
       <c r="B39" s="4" t="n"/>
@@ -2095,7 +2095,11 @@
       <c r="L39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Reading: the control configurations are statistically indistinguishable between v1 and v2 at the 5 % level. With 6 configurations, the sign test can detect only large systematic shifts. The LLM is not seeded, so run-to-run variation alone also differs between versions.</t>
+        </is>
+      </c>
       <c r="B40" s="4" t="n"/>
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="4" t="n"/>
@@ -2109,11 +2113,7 @@
       <c r="L40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Control check v2 → v3</t>
-        </is>
-      </c>
+      <c r="A41" s="4" t="n"/>
       <c r="B41" s="4" t="n"/>
       <c r="C41" s="4" t="n"/>
       <c r="D41" s="4" t="n"/>
@@ -2127,9 +2127,9 @@
       <c r="L41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Sign test over the 6 configurations: 4 differ, 2 of them higher in v3; two-sided p = 1.000.</t>
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Control check v2 → v3</t>
         </is>
       </c>
       <c r="B42" s="4" t="n"/>
@@ -2147,7 +2147,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Pooled run-level Fisher exact test: 20/30 in v2 vs 21/30 in v3; p = 1.000.</t>
+          <t>Sign test over the 6 configurations: 4 differ, 2 of them higher in v3; two-sided p = 1.000.</t>
         </is>
       </c>
       <c r="B43" s="4" t="n"/>
@@ -2165,7 +2165,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Reading: the control configurations are statistically indistinguishable between v2 and v3 at the 5 % level. Unlike v1 → v2, the v3 changes can act on these configurations too (rejected mismatched modifications, id-stem mapping, best-iteration order), so this is a check that they did not shift them, not a pure null comparison. With 6 configurations the sign test detects only large systematic shifts; the LLM is not seeded, so run-to-run variation also differs between batches.</t>
+          <t>Pooled run-level Fisher exact test: 20/30 in v2 vs 21/30 in v3; p = 1.000.</t>
         </is>
       </c>
       <c r="B44" s="4" t="n"/>
@@ -2180,20 +2180,39 @@
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="n"/>
     </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Reading: the control configurations are statistically indistinguishable between v2 and v3 at the 5 % level. Unlike v1 → v2, the v3 changes can act on these configurations too (rejected mismatched modifications, id-stem mapping, best-iteration order), so this is a check that they did not shift them, not a pure null comparison. With 6 configurations the sign test detects only large systematic shifts; the LLM is not seeded, so run-to-run variation also differs between batches.</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>